<commit_message>
Initial commit of AI summarisor project
</commit_message>
<xml_diff>
--- a/backend/storage/history.xlsx
+++ b/backend/storage/history.xlsx
@@ -466,22 +466,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ce9e02b7-7947-40dc-946a-3ebc825afc01</t>
+          <t>3c4b2d08-4702-4298-bfbd-358269bd74e5</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ranjithagowda9801@gmail.com</t>
+          <t>sahanashaiva01@gmail.com</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Revised_AI_MultiSummarizer_Plan (1).pdf</t>
+          <t>https://www.nasa.gov/humans-in-space/artemis</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>file</t>
+          <t>url</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -491,44 +491,44 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>The project aims to create a sophisticated full-stack application that can extract, clean, and summarize text from vario...</t>
+          <t xml:space="preserve">The Artemis program is a series of missions that will enable human exploration at the Moon and future missions to Mars. </t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>["AI", "Summarizer", "Content Intelligence", "React"]</t>
+          <t>["Artemis", "NASA", "Moon", "Mars"]</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>{"summary_concise": "The project involves developing a multi-format AI summarizer that can process diverse content sources, including URLs and documents, and provide sentiment analysis and reading metrics.", "summary_detailed": "The project aims to create a sophisticated full-stack application that can extract, clean, and summarize text from various sources using AI. The system will provide sentiment analysis and reading metrics in a modern dashboard. The application will have a modular grid UI, with each card having a specific responsibility, such as input module, metrics, main output, and visuals. The project will be implemented in several stages, including multi-source extraction, NLP core, API development, React Bento layout, and integration and analytics. The application will use various technologies, including React, Python, FastAPI, and NLTK. The project will also involve implementing a sentiment chart and a history sidebar to save past results.", "key_points": ["Multi-format AI summarizer", "Diverse content sources", "Sentiment analysis and reading metrics", "Modular grid UI", "Multi-stage implementation"], "important_insights": ["The application will use AI to extract and summarize text from various sources", "The system will provide sentiment analysis and reading metrics", "The UI will be modular and grid-based", "The project will involve multiple stages of implementation"], "keywords": ["AI", "Summarizer", "Content Intelligence", "React", "Python", "NLTK"], "metadata_insights": {"detected_topic": "Artificial Intelligence", "reading_difficulty": "Advanced", "content_complexity": "High", "estimated_audience": "Technical professionals", "category": "Technology", "writing_style": "Technical"}, "tone_analysis": {"overall_tone": "Informative", "sentiment": "Neutral", "formality": "Formal", "confidence": "High", "confidence_score": 90, "sentiment_scores": {"positive": 10, "negative": 0, "neutral": 90}}, "source_text": "Multi-Format AI Summarizer\nAdvanced Content Intelligence Platform (URL, PDF, DOCX)\nProject Scope\nA sophisticated full-stack application that processes diverse content sources. Whether a\nuser provides a website link or uploads a document (PDF/Word), the system extracts,\ncleans, and summarizes the text using AI, providing sentiment analysis and reading\nmetrics in a modern dashboard.\nTechnical Requirements\nFrontend (React) Backend (Python)\n- React.js (Hooks &amp; Context) - FastAPI or Flask (REST API)\n- Tailwind CSS (Bento Layout) - PyPDF2 / pdfplumber (PDF)\n- React-Dropzone (File Uploads) - python-docx (Word Docs)\n- Recharts (Data Visuals) - BeautifulSoup4 (URL Scraping)\nAI &amp; Processing Workflow\n- NLTK / TextBlob (Summarization) - Axios for HTTP Requests\n- VADER (Sentiment Analysis) - FormData for File uploads\n- LangChain (Optional for better - LocalStorage for History\nchains)\nUI Design: Bento Dashboard\nThe UI is organized into a modular grid. Each \"card\" has a specific responsibility:\nInput Module: URL Toggle &amp; Drag-and-Drop File Zone\nMetrics: Word Count &amp; Read Time Main Output: AI\nGenerated Summary\n(Bulleted)\nVisuals: Sentiment Donut Chart\nImplementation Roadmap\n1 Multi-Source Extraction: Build a Python utility class that accepts a source (URL or\nFile). Use conditional logic to trigger the correct parser (BS4 for URLs, pdfplumber\nfor PDFs).\n2 NLP Core: Implement the summarization engine. Ensure the output is structured\n(Title, Key Points, Tone) so the React frontend can map it easily to cards.\n3 API Development: Create a POST endpoint that handles both JSON (for URLs) and\nMultipart/Form-Data (for file uploads).\n4 React Bento Layout: Build the grid using Tailwind `grid-cols`. Create a stateful\n\"Input Card\" that changes its UI based on whether the user wants to paste a link or\nupload a file.\n5 Integration &amp; Analytics: Connect the UI to the API. Implement the Sentiment\nChart and the history sidebar to save past results.\n"}</t>
+          <t>{"summary_concise": "NASA's Artemis program aims to return humans to the Moon and eventually send them to Mars, with a focus on scientific discovery, economic benefits, and inspiration for future generations.", "summary_detailed": "The Artemis program is a series of missions that will enable human exploration at the Moon and future missions to Mars. The program includes the development of the Space Launch System (SLS) rocket, the Orion spacecraft, and the Gateway, a small space station that will serve as a multi-purpose outpost supporting lunar surface missions. The program also involves the development of human landing systems, or next-generation landers, that will safely carry Artemis astronauts from lunar orbit to the Moon's surface and back. The Artemis Accords, established in 2020, provide a common set of principles to enhance the governance of the civil exploration and use of outer space. The program has already achieved several milestones, including the launch of the Artemis I mission, which sent the Orion spacecraft on a 1.4-million-mile journey beyond the Moon and back.", "key_points": ["NASA's Artemis program aims to return humans to the Moon and eventually send them to Mars", "The program includes the development of the Space Launch System (SLS) rocket and the Orion spacecraft", "The Gateway, a small space station, will serve as a multi-purpose outpost supporting lunar surface missions", "The Artemis Accords provide a common set of principles to enhance the governance of the civil exploration and use of outer space"], "important_insights": ["The Artemis program is a crucial step towards establishing a sustainable human presence on the Moon and eventually sending humans to Mars", "The program involves international cooperation and the development of new technologies and systems", "The Artemis Accords provide a framework for responsible and sustainable exploration and use of outer space"], "keywords": ["Artemis", "NASA", "Moon", "Mars", "Space Exploration", "Gateway", "Orion", "SLS"], "metadata_insights": {"detected_topic": "Space Exploration", "reading_difficulty": "Intermediate", "content_complexity": "High", "estimated_audience": "General Audience", "category": "Science and Technology", "writing_style": "Informative"}, "tone_analysis": {"overall_tone": "Informative", "sentiment": "Neutral", "formality": "Formal", "confidence": "High", "confidence_score": 90, "sentiment_scores": {"positive": 20, "negative": 0, "neutral": 80}}, "source_text": "Moon to Mars | NASA's Artemis Program - NASA\nSearch\nSuggested Searches\nClimate Change\nArtemis\nExpedition 64\nMars perseverance\nSpaceX Crew-2\nInternational Space Station\nView All Topics A-Z\nHome\nMissions\nHumans in Space\nEarth\nThe Solar System\nThe Universe\nScience\nAeronautics\nTechnology\nLearning Resources\nAbout NASA\nEspa\u00f1ol\nNews &amp; Events\nMultimedia\nNASA+\nFeatured\n3 min read\nNASA\u2019s Simulated Mars Mission Marks 200 Days Inside Habitat\narticle\n5 days ago\n6 min read\nNASA Pushes Next-Gen Mars Helicopter Rotor Blades Past Mach 1\narticle\n5 days ago\n3 min read\nWhat\u2019s Up: May 2026 Skywatching Tips from NASA\narticle\n2 weeks ago\nBack\nMissions\nSearch All NASA Missions\nA to Z List of Missions\nUpcoming Launches and Landings\nSpaceships and Rockets\nCommunicating with Missions\nArtemis\nJames Webb Space Telescope\nHubble Space Telescope\nInternational Space Station\nOSIRIS-Rex\nHumans in Space\nWhy Go to Space\nAstronauts\nCommercial Space\nDestinations\nSpaceships and Rockets\nLiving in Space\nEarth\nExplore Earth Science\nClimate Change\nEarth, Our Planet\nEarth Science in Action\nEarth Multimedia\nEarth Data\nEarth Science Researchers\nThe Solar System\nThe Sun\nMercury\nVenus\nEarth\nThe Moon\nMars\nJupiter\nSaturn\nUranus\nNeptune\nPluto &amp; Dwarf Planets\nAsteroids, Comets &amp; Meteors\nThe Kuiper Belt\nThe Oort Cloud\nSkywatching\nThe Universe\nExoplanets\nThe Search for Life in the Universe\nStars\nGalaxies\nBlack Holes\nThe Big Bang\nDark Energy\nDark Matter\nScience\nEarth Science\nPlanetary Science\nAstrophysics &amp; Space Science\nThe Sun &amp; Heliophysics\nBiological &amp; Physical Sciences\nLunar Science\nCitizen Science\nAstromaterials\nAeronautics Research\nHuman Space Travel Research\nAeronautics\nScience in the Air\nNASA Aircraft\nFlight Research Innovation\nSupersonic Flight\nAir Traffic Solutions\nGreen Aviation Tech\nDrones &amp; You\nTechnology\nTechnology Transfer &amp; Spinoffs\nSpace Travel Technology\nTechnology Living in Space\nManufacturing and Materials\nRobotics\nScience Instruments\nComputing\nLearning Resources\nFor Kids and Students\nFor Educators\nFor Colleges and Universities\nFor Professionals\nScience for Everyone\nRequests for Exhibits, Artifacts, Speakers &amp; Flyovers\nSTEM Engagement at NASA\nAbout NASA\nNASA's Impacts\nCenters and Facilities\nDirectorates\nOrganizations\nPeople of NASA\nCareers\nInternships\nOur History\nDoing Business with NASA\nGet Involved\nContact\nNASA en Espa\u00f1ol\nCiencia\nAeron\u00e1utica\nCiencias Terrestres\nSistema Solar\nUniverso\nNews &amp; Events\nNews Releases\nRecently Published\nVideo Series on NASA+\nPodcasts &amp; Audio\nBlogs\nNewsletters\nSocial Media\nMedia Resources\nEvents\nUpcoming Launches &amp; Landings\nVirtual Guest Program\nMultimedia\nNASA+\nImages\nNASA Live\nNASA Apps\nPodcasts\nImage of the Day\ne-Books\nInteractives\nSTEM Multimedia\nNASA Brand &amp; Usage Guidelines\nFeatured\n3 min read\nIndustry Moon Lander Training Cabin Lands at NASA for Artemis\narticle\n5 days ago\n3 min read\nNASA\u2019s Simulated Mars Mission Marks 200 Days Inside Habitat\narticle\n5 days ago\n5 min read\nNASA\u2019s Roman Poised to Transform Hunt for Elusive Neutron Stars\narticle\n6 days ago\nHighlights\n3 min read\nNASA\u2019s Simulated Mars Mission Marks 200 Days Inside Habitat\narticle\n5 days ago\n2 min read\nNASA Astronaut to Answer Questions from Students in Florida\narticle\n7 days ago\n4 min read\nLiquid Lifeline: NASA Tech Could Create IV Fluid In Space\narticle\n3 weeks ago\nHighlights\n3 min read\nAustralia\u2019s Cloudy Beauty\narticle\n13 hours ago\n2 min read\nMay 2026 Satellite Puzzler\narticle\n19 hours ago\n4 min read\nTracy Arm\u2019s Post-Tsunami Landscape\narticle\n5 days ago\nHighlights\n6 min read\nNASA\u2019s Perseverance Rover Snaps Selfie in Mars\u2019 Western Frontier\narticle\n3 minutes ago\n6 min read\nNASA Pushes Next-Gen Mars Helicopter Rotor Blades Past Mach 1\narticle\n5 days ago\n3 min read\nNew NASA HEAT Coloring Book Blends Art, Science, and Cultural Perspectives\narticle\n1 week ago\nFeatured\n7 min read\nHubble Survey Sets Up Roman\u2019s Future Look Near Milky Way\u2019s Center\narticle\n1 day ago\n5 min read\nNASA\u2019s Roman Poised to Transform Hunt for Elusive Neutron Stars\narticle\n6 days ago\n4 min read\nFor NASA\u2019s TESS, Stellar Eclipses Shed Light on Possible New Worlds\narticle\n1 week ago\nHighlights\n2 min read\nODYSSEY:\u00a0NASA\u00a0Analyzing\u00a0Bacteria in\u00a0Space, Simulated\u00a0Microgravity\narticle\n3 hours ago\n3 min read\nJoint Earth Observation Mission Quality Assessment Framework \u2013 Optical Guidelines Documents Released\narticle\n22 hours ago\n7 min read\nHubble Survey Sets Up Roman\u2019s Future Look Near Milky Way\u2019s Center\narticle\n1 day ago\nHighlights\n3 min read\nMeet the Fleet: NASA Armstrong Continues Legacy of Flight Research\narticle\n5 days ago\n6 min read\nCornell Students Aid NASA with Drone Safety in Sky\narticle\n5 days ago\n4 min read\nD-Site\narticle\n1 week ago\nHighlights\n4 min read\nHello Universe: NASA\u2019s Next-Gen Space Processor Undergoes Testing\narticle\n2 hours ago\n3 min read\nI Am Artemis: Kathleen Harmon\narticle\n2 hours ago\n1 min read\nAmendment 56: D.6 APRA and D.7 SAT Final Text and Due Dates\narticle\n4 days ago\nFeatured\n4 min read\nSpace Out This Summer with Variety of NASA STEM Activities\narticle\n2 weeks ago\nFeatured\n3 min read\nNASA, Industry Advance High Performance Spaceflight Computing\narticle\n4 days ago\n4 min read\nNASA Fuel Cell Tests Pave Way for Energy Storage on Moon\narticle\n4 days ago\n3 min read\nNASA Welcomes Paraguay as 67th Artemis Accords Signatory\narticle\n5 days ago\nHighlights\n11 min read\nLa NASA anuncia la cobertura de la misi\u00f3n lunar Artemis II\narticle\n2 months ago\n15 min read\nAgenda diaria de la misi\u00f3n a la Luna de Artemis\u00a0II de la NASA\narticle\n2 months ago\n6 min read\nLa NASA refuerza Artemis: a\u00f1ade una misi\u00f3n y perfecciona su arquitectura general\narticle\n2 months ago\nArtemis\nArtemis\nUnder Artemis, NASA will send astronauts on increasingly difficult missions to explore more of the Moon for scientific discovery, economic benefits, and to build on our foundation for the first crewed missions to Mars.\nQuick Facts\nArtemis II, the first crewed Artemis flight, marks a key step toward long\u2011term return to the Moon and future missions to Mars.\nDuring Artemis I, the SLS (Space Launch System), roared into the night sky and sent the Orion spacecraft on a 1.4-million-mile journey beyond the Moon and back.\nNASA, in coordination with the U.S. Department of State and seven other initial signatory nations, established the Artemis Accords in 2020.\nStrengthening Artemis\nTo achieve the national goal of landing American astronauts on the surface of the Moon and maintaining U.S. superiority in exploration and discovery, NASA is increasing its cadence of missions under the Artemis program, standardizing the SLS (Space Launch System) rocket configuration, and adding a new mission.\nArtemis Missions\nabout Strengthening Artemis\nArtemis News\nMore Artemis News\nArticle\n3 Min Read\nI Am Artemis: Kathleen Harmon\nArticle\n2 Min Read\nNicholas Houghton: Engineering Crew Safety for NASA\u2019s Artemis Missions\nArticle\n3 Min Read\nI Am Artemis: Anton Kiriwas\nArticle\n4 Min Read\nNASA Fuel Cell Tests Pave Way for Energy Storage on Moon\n61 Min Read\nArtemis II: Backup Crew\n3 Min Read\nNASA Welcomes Paraguay as 67th Artemis Accords Signatory\nArticle\n3 Min Read\nIndustry Moon Lander Training Cabin Lands at NASA for Artemis\nArticle\n3 Min Read\nNASA Welcomes Ireland as Newest Artemis Accords Signatory\nArticle\nLunar Exploration\nLunar Discovery\nMoon to Mars\nLunar Exploration\nThe Moon is a 4.5-billion-year-old time capsule.\nWe\u2019re going back to the Moon for scientific discovery, economic benefits, and inspiration for a new generation of explorers. While maintaining American leadership in exploration, we will build a global alliance and explore deep space for the benefit of all.\nEarth's Moon\nOn flight day six of the Artemis I mission, the Orion spacecraft used its optical navigation camera to snap this black-and-white photo of the Moon.\nNASA\nLunar Discovery\nThe Moon holds clues to the evolution of Earth, the planets, and the Sun.\nThrough Artemis, NASA will address high priority science questions, focusing on those that are best accomplished by on-site human explorers on and around the Moon and Mars by using robotic surface and orbiting systems.\nArtemis Science\nArtemis geology training lead at Johnson Space Center in Houston, Cindy Evans (left) and NASA astronaut Christina Koch study geologic features in Iceland during Artemis II crew geology training in August 2024.\nNASA/Robert Markowitz\nMoon to Mars\nLike the Moon, Mars is a rich destination for scientific discovery.\nMars remains our horizon goal for human exploration because it is one of the only other places we know where life may have existed in the solar system. What we learn about the Red Planet will tell us more about our Earth\u2019s past and future, and may help answer whether life exists beyond our home planet.\nHumans on Mars\nIllustration of an astronaut on Mars using a remote control drone to inspect a nearby cliff.\nNASA\nMissions\nArtemis I\nLaunched in 2022, Artemis I was the first in a series of increasingly complex missions that will enable human exploration at the Moon and future missions to Mars.\nArtemis II\nThe first crewed Artemis flight marks a key step toward long\u2011term return to the Moon and future missions to Mars.\nArtemis III\nScheduled for 2027, this new demonstration mission in low Earth orbit will test one or both commercial landers from SpaceX and Blue Origin, respectively.\nArtemis IV\nNASA continues to target early 2028 for the first Artemis lunar landing, a date that has remained unchanged since mid\u20112025. After reaching lunar orbit, the crew will transfer from Orion to a commercial lunar lander for their descent to the Moon\u2019s surface.\nArtemis V\nUsing the standard SLS (Space Launch System) rocket configuration, NASA expects to launch this lunar surface mission by late 2028, with subsequent missions planned roughly once per year.\nOur Artemis II Crew\nMeet the astronauts who ventured around the Moon on Artemis II, the first crewed flight aboard NASA\u2019s human deep space capabilities, paving the way for future lunar surface missions.\nForging New Frontiers\nabout Our Artemis II Crew\nMedia Resources\nArtemis II Press Kit\nArtemis II Reference Guide\nArtemis II Resources for Media\nSpacecraft\nRocket\nGround Systems\nLunar Landers\nSpacesuits &amp; Rovers\nLunar Delivery\nGateway\nArtemis Partners\nCarrying Humanity to the Moon\nOrion is developed to be capable of sending astronauts to the Moon and is a crucial step toward eventually sending crews on to Mars.\nThe Orion spacecraft will serve as the exploration vehicle that will carry and sustain the crew on Artemis missions to the Moon and return them safely to Earth. Orion will launch on NASA\u2019s new heavy-lift rocket, the SLS (Space Launch System).\nAbout Orion\nThe full Moon is seen behind NASA\u2019s Artemis II SLS (Space Launch System) rocket and Orion spacecraft, standing atop a mobile launcher at Launch Complex 39B, Sunday, Feb. 1, 2026, at Kennedy Space Center in Florida.\nNASA/John Kraus\nA Single Launch\nNASA\u2019s Space Launch System (SLS) offers more payload mass, volume, and departure energy than any other single rocket.\nCombining power and capability, NASA\u2019s SLS (Space Launch System) rocket is part of NASA\u2019s backbone for deep space exploration and Artemis. SLS is the only rocket that can send Orion, astronauts, and cargo directly to the Moon in a single launch.\nAbout the Space Launch System\nClouds and the Sun illuminate the sky on Wednesday, Jan. 28, 2026, as NASA\u2019s Artemis II SLS (Space Launch System) rocket and Orion spacecraft stand vertical at Launch Complex 39B at Kennedy Space Center in Florida.\nNASA/Cory S. Huston\nThe Infrastructure\nPreparing the infrastructure to support NASA\u2019s SLS (Space Launch System) rocket and Orion spacecraft.\nExploration Ground Systems, based at Kennedy Space Center in Florida, develops and operates the systems and facilities needed to process, launch, and recover rockets and spacecraft for NASA\u2019s Artemis missions.\nAbout Exploration Ground Systems\nTechnicians with NASA\u2019s Exploration Ground Systems team prepare to attach a crane to lift and secure NASA\u2019s Orion spacecraft on top of the SLS (Space Launch System) rocket in High Bay 3 of the Vehicle Assembly Building at Kennedy Space Center in Florida on Friday, Oct. 17, 2025.\nNASA/Amber Jean Notvest\nDelivering Crew, Cargo to the Lunar Frontier\nWorking with American industry to send crew, cargo, and supplies to the Moon.\nNASA is working with industry to develop the human landing systems, or next-generation landers, that will safely carry Artemis astronauts from lunar orbit to the\u2002Moon\u2019s surface and back for future crewed exploration of the Moon.\nAbout Lunar Landers\nArtist concept of SpaceX\u2019s Starship Human Landing System (HLS) on the Moon.\nSpaceX\nMobility for Every Mission\nProviding spacesuit capabilities and surface mobility systems for humanity\u2019s return to the Moon.\nThe Extravehicular Activity and Human Surface Mobility Program serves as NASA\u2019s program to develop next-generation spacesuits, human-rated rovers, tools, and the spacewalk support systems that will enable astronauts to survive and work outside the confines of a spacecraft to explore on and around the Moon.\nAbout Spacesuits &amp; Rovers\nIllustration of Artemis astronauts working on the Moon.\nNASA\nLanding on the Moon\nWorking with American companies to deliver science and technology to the Moon\u2019s surface.\nThe Commercial Lunar Payload Services (CLPS) initiative allows rapid acquisition of lunar delivery services from commercial vendors to send NASA science and technology payloads, enabling industry growth and supporting long-term lunar exploration. The CLPS model offers a unique opportunity to test and refine technologies and integrate systems that will provide insight for future crewed missions to the Moon.\nAbout Commercial Lunar Payload Services\nCarrying a suite of NASA science and technology, Firefly Aerospace\u2019s Blue Ghost Mission 1 successfully landed at 3:34 a.m. EST on Sunday, March 2, 2025, near a volcanic feature called Mons Latreille within Mare Crisium, a more than 300-mile-wide basin located in the northeast quadrant of the Moon\u2019s near side.\nFirefly Aerospace\nDeep Space Exploration\nHumanity\u2019s first space station around the Moon.\nGateway is central to the NASA-led Artemis missions to return to the Moon for scientific discovery and chart a path for the first human missions to Mars and beyond. The small space station will be a multi-purpose outpost supporting lunar surface missions, science in lunar orbit, and human exploration further into the cosmos.\nAbout Gateway\nGateway\u2019s HALO (Habitation and Logistics Outpost) at Northrop Grumman\u2019s facility in Gilbert, Arizona, on April 4, 2025, shortly after its arrival from Thales Alenia Space in Turin, Italy.\nNASA/Josh Valcarcel\nA Lunar Economy\nMen and women across America and around the world are building the systems to support missions to the Moon, Mars, and beyond.\nSince its inception, every state in America has made a contribution to the success of NASA\u2019s Artemis campaign, with companies hard at work on innovations that will help establish a long-term human presence at the Moon. These missions are critical to an expanding space economy, fueling new industries and technologies, supporting job growth, and furthering the demand for a highly skilled workforce.\nAbout Artemis Partners\nNASA\u2019s Artemis II Space Launch System (SLS) rocket and Orion spacecraft, secured to the mobile launcher, make the 4.2 mile journey toward Launch Pad 39B, Saturday, Jan. 17, 2026, at Kennedy Space Center in Florida.\nNASA/Keegan Barber\nThe Artemis Accords\nNASA, in coordination with the U.S. Department of State and seven other initial signatory nations, established the Artemis Accords in 2020. Now with more than 60 signatories, the Artemis Accords provide a common set of principles to enhance the governance of the civil exploration and use of outer space as many countries and private companies conduct missions and operations around the Moon.\nCivil Space Exploration\nabout The Artemis Accords\nLearning Resources\nJoin Artemis\nFind your place in space.\nMake, launch, compete and learn. Find your favorite way to be part of the Artemis mission.\nStart Exploring\nabout Join Artemis\nKeep Exploring\nDiscover More\nHumans In Space\nDestinations\nAstronauts\nLiving in Space\nWas this page helpful?\n\u0394\nWas this page helpful?\nYes\nNo\n\u00d7"}</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-05-08T22:23:36.765368</t>
+          <t>2026-05-12T21:02:06.909847</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>de3876b5-187a-4bd8-9029-233c986d6377</t>
+          <t>d2024d82-eb9c-4122-9f7d-9c2fc20e837a</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ranjithagowda9801@gmail.com</t>
+          <t>sahanasahana40163@gmail.com</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Revised_AI_MultiSummarizer_Plan (1).pdf</t>
+          <t>https://www.nasa.gov/humans-in-space/artemis</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>file</t>
+          <t>url</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -538,44 +538,44 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>The application is designed to handle multiple content sources, including URLs and documents, and utilizes a range of te...</t>
+          <t xml:space="preserve">The Artemis program is a series of missions that will enable human exploration at the Moon and future missions to Mars. </t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>["AI Summarizer", "Content Intelligence", "Natural Language Processing", "React"]</t>
+          <t>["Artemis", "NASA", "Moon", "Mars"]</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>{"summary_concise": "The Multi-Format AI Summarizer is a full-stack application that processes diverse content sources, extracting, cleaning, and summarizing text using AI, and providing sentiment analysis and reading metrics.", "summary_detailed": "The application is designed to handle multiple content sources, including URLs and documents, and utilizes a range of technologies such as React, Python, and natural language processing libraries to provide a comprehensive summary and analysis of the input text. The system consists of several components, including a frontend built with React, a backend built with Python, and a range of libraries and tools for tasks such as sentiment analysis and data visualization. The application is implemented in several stages, including multi-source extraction, NLP core implementation, API development, and integration with the React frontend. The final product provides a modern dashboard with features such as a modular grid, input module, metrics, and visualizations. The application is designed to be user-friendly and provides a range of features to facilitate the analysis and understanding of complex text data.", "key_points": ["Multi-format support for URLs and documents", "AI-powered text summarization and sentiment analysis", "Modern dashboard with modular grid and data visualizations", "Implementation in several stages, including frontend and backend development", "Utilization of a range of technologies and libraries, including React and Python"], "important_insights": ["The application is designed to handle diverse content sources and provide comprehensive analysis and summary", "The use of AI and natural language processing libraries enables advanced text analysis and sentiment detection", "The modular grid design and data visualizations provide a user-friendly interface for exploring and understanding complex text data", "The application is implemented in several stages, allowing for a phased approach to development and testing"], "keywords": ["AI Summarizer", "Content Intelligence", "Natural Language Processing", "React", "Python", "Sentiment Analysis"], "metadata_insights": {"detected_topic": "Artificial Intelligence and Natural Language Processing", "reading_difficulty": "Advanced", "content_complexity": "High", "estimated_audience": "Technical professionals and developers", "category": "Technology and Software Development", "writing_style": "Technical and Informative"}, "tone_analysis": {"overall_tone": "Informative", "sentiment": "Neutral", "formality": "Formal", "confidence": "High", "confidence_score": 90, "sentiment_scores": {"positive": 10, "negative": 0, "neutral": 90}}, "source_text": "Multi-Format AI Summarizer\nAdvanced Content Intelligence Platform (URL, PDF, DOCX)\nProject Scope\nA sophisticated full-stack application that processes diverse content sources. Whether a\nuser provides a website link or uploads a document (PDF/Word), the system extracts,\ncleans, and summarizes the text using AI, providing sentiment analysis and reading\nmetrics in a modern dashboard.\nTechnical Requirements\nFrontend (React) Backend (Python)\n- React.js (Hooks &amp; Context) - FastAPI or Flask (REST API)\n- Tailwind CSS (Bento Layout) - PyPDF2 / pdfplumber (PDF)\n- React-Dropzone (File Uploads) - python-docx (Word Docs)\n- Recharts (Data Visuals) - BeautifulSoup4 (URL Scraping)\nAI &amp; Processing Workflow\n- NLTK / TextBlob (Summarization) - Axios for HTTP Requests\n- VADER (Sentiment Analysis) - FormData for File uploads\n- LangChain (Optional for better - LocalStorage for History\nchains)\nUI Design: Bento Dashboard\nThe UI is organized into a modular grid. Each \"card\" has a specific responsibility:\nInput Module: URL Toggle &amp; Drag-and-Drop File Zone\nMetrics: Word Count &amp; Read Time Main Output: AI\nGenerated Summary\n(Bulleted)\nVisuals: Sentiment Donut Chart\nImplementation Roadmap\n1 Multi-Source Extraction: Build a Python utility class that accepts a source (URL or\nFile). Use conditional logic to trigger the correct parser (BS4 for URLs, pdfplumber\nfor PDFs).\n2 NLP Core: Implement the summarization engine. Ensure the output is structured\n(Title, Key Points, Tone) so the React frontend can map it easily to cards.\n3 API Development: Create a POST endpoint that handles both JSON (for URLs) and\nMultipart/Form-Data (for file uploads).\n4 React Bento Layout: Build the grid using Tailwind `grid-cols`. Create a stateful\n\"Input Card\" that changes its UI based on whether the user wants to paste a link or\nupload a file.\n5 Integration &amp; Analytics: Connect the UI to the API. Implement the Sentiment\nChart and the history sidebar to save past results.\n"}</t>
+          <t>{"summary_concise": "NASA's Artemis program aims to send astronauts to the Moon and eventually to Mars, with a focus on scientific discovery, economic benefits, and inspiration for a new generation of explorers.", "summary_detailed": "The Artemis program is a series of missions that will enable human exploration at the Moon and future missions to Mars. The program includes the development of the Space Launch System (SLS) rocket, the Orion spacecraft, and the Gateway, a small space station that will be a multi-purpose outpost supporting lunar surface missions. The Artemis program also involves the development of new technologies, such as next-generation spacesuits and human-rated rovers, to enable astronauts to survive and work outside the confines of a spacecraft. The program has already achieved several milestones, including the launch of the Artemis I mission, which sent the Orion spacecraft on a 1.4-million-mile journey beyond the Moon and back. The Artemis II mission, the first crewed Artemis flight, is scheduled to launch in the near future, marking a key step toward long-term return to the Moon and future missions to Mars.", "key_points": ["NASA's Artemis program aims to send astronauts to the Moon and eventually to Mars", "The program includes the development of the Space Launch System (SLS) rocket and the Orion spacecraft", "The Gateway, a small space station, will be a multi-purpose outpost supporting lunar surface missions", "The program involves the development of new technologies, such as next-generation spacesuits and human-rated rovers", "The Artemis II mission, the first crewed Artemis flight, is scheduled to launch in the near future"], "important_insights": ["The Artemis program is a critical step towards establishing a sustainable human presence on the Moon and eventually on Mars", "The program has the potential to drive innovation and economic growth, as well as inspire a new generation of scientists, engineers, and explorers", "The development of new technologies and capabilities through the Artemis program will have far-reaching implications for space exploration and beyond"], "keywords": ["Artemis", "NASA", "Moon", "Mars", "Space Exploration", "Space Launch System", "Orion Spacecraft", "Gateway"], "metadata_insights": {"detected_topic": "Space Exploration", "reading_difficulty": "Intermediate", "content_complexity": "High", "estimated_audience": "General Audience", "category": "Science and Technology", "writing_style": "Informative"}, "tone_analysis": {"overall_tone": "Informative", "sentiment": "Neutral", "formality": "Formal", "confidence": "High", "confidence_score": 90, "sentiment_scores": {"positive": 40, "negative": 10, "neutral": 50}}, "source_text": "Moon to Mars | NASA's Artemis Program - NASA\nSearch\nSuggested Searches\nClimate Change\nArtemis\nExpedition 64\nMars perseverance\nSpaceX Crew-2\nInternational Space Station\nView All Topics A-Z\nHome\nMissions\nHumans in Space\nEarth\nThe Solar System\nThe Universe\nScience\nAeronautics\nTechnology\nLearning Resources\nAbout NASA\nEspa\u00f1ol\nNews &amp; Events\nMultimedia\nNASA+\nFeatured\n6 min read\nNASA\u2019s Perseverance Rover Snaps Selfie in Mars\u2019 Western Frontier\narticle\n11 hours ago\n6 min read\nNASA Pushes Next-Gen Mars Helicopter Rotor Blades Past Mach 1\narticle\n5 days ago\n3 min read\nWhat\u2019s Up: May 2026 Skywatching Tips from NASA\narticle\n2 weeks ago\nBack\nMissions\nSearch All NASA Missions\nA to Z List of Missions\nUpcoming Launches and Landings\nSpaceships and Rockets\nCommunicating with Missions\nArtemis\nJames Webb Space Telescope\nHubble Space Telescope\nInternational Space Station\nOSIRIS-Rex\nHumans in Space\nWhy Go to Space\nAstronauts\nCommercial Space\nDestinations\nSpaceships and Rockets\nLiving in Space\nEarth\nExplore Earth Science\nClimate Change\nEarth, Our Planet\nEarth Science in Action\nEarth Multimedia\nEarth Data\nEarth Science Researchers\nThe Solar System\nThe Sun\nMercury\nVenus\nEarth\nThe Moon\nMars\nJupiter\nSaturn\nUranus\nNeptune\nPluto &amp; Dwarf Planets\nAsteroids, Comets &amp; Meteors\nThe Kuiper Belt\nThe Oort Cloud\nSkywatching\nThe Universe\nExoplanets\nThe Search for Life in the Universe\nStars\nGalaxies\nBlack Holes\nThe Big Bang\nDark Energy\nDark Matter\nScience\nEarth Science\nPlanetary Science\nAstrophysics &amp; Space Science\nThe Sun &amp; Heliophysics\nBiological &amp; Physical Sciences\nLunar Science\nCitizen Science\nAstromaterials\nAeronautics Research\nHuman Space Travel Research\nAeronautics\nScience in the Air\nNASA Aircraft\nFlight Research Innovation\nSupersonic Flight\nAir Traffic Solutions\nGreen Aviation Tech\nDrones &amp; You\nTechnology\nTechnology Transfer &amp; Spinoffs\nSpace Travel Technology\nTechnology Living in Space\nManufacturing and Materials\nRobotics\nScience Instruments\nComputing\nLearning Resources\nFor Kids and Students\nFor Educators\nFor Colleges and Universities\nFor Professionals\nScience for Everyone\nRequests for Exhibits, Artifacts, Speakers &amp; Flyovers\nSTEM Engagement at NASA\nAbout NASA\nNASA's Impacts\nCenters and Facilities\nDirectorates\nOrganizations\nPeople of NASA\nCareers\nInternships\nOur History\nDoing Business with NASA\nGet Involved\nContact\nNASA en Espa\u00f1ol\nCiencia\nAeron\u00e1utica\nCiencias Terrestres\nSistema Solar\nUniverso\nNews &amp; Events\nNews Releases\nRecently Published\nVideo Series on NASA+\nPodcasts &amp; Audio\nBlogs\nNewsletters\nSocial Media\nMedia Resources\nEvents\nUpcoming Launches &amp; Landings\nVirtual Guest Program\nMultimedia\nNASA+\nImages\nNASA Live\nNASA Apps\nPodcasts\nImage of the Day\ne-Books\nInteractives\nSTEM Multimedia\nNASA Brand &amp; Usage Guidelines\nFeatured\n6 min read\nNASA\u2019s Perseverance Rover Snaps Selfie in Mars\u2019 Western Frontier\narticle\n11 hours ago\n3 min read\nNASA\u2019s Simulated Mars Mission Marks 200 Days Inside Habitat\narticle\n6 days ago\n7 min read\nHubble Survey Sets Up Roman\u2019s Future Look Near Milky Way\u2019s Center\narticle\n2 days ago\nHighlights\n3 min read\nNASA\u2019s Simulated Mars Mission Marks 200 Days Inside Habitat\narticle\n6 days ago\n2 min read\nNASA Astronaut to Answer Questions from Students in Florida\narticle\n1 week ago\n4 min read\nLiquid Lifeline: NASA Tech Could Create IV Fluid In Space\narticle\n3 weeks ago\nHighlights\n3 min read\nAustralia\u2019s Cloudy Beauty\narticle\n24 hours ago\n2 min read\nMay 2026 Satellite Puzzler\narticle\n1 day ago\n4 min read\nTracy Arm\u2019s Post-Tsunami Landscape\narticle\n5 days ago\nHighlights\n6 min read\nNASA\u2019s Perseverance Rover Snaps Selfie in Mars\u2019 Western Frontier\narticle\n11 hours ago\n6 min read\nNASA Pushes Next-Gen Mars Helicopter Rotor Blades Past Mach 1\narticle\n5 days ago\n3 min read\nNew NASA HEAT Coloring Book Blends Art, Science, and Cultural Perspectives\narticle\n1 week ago\nFeatured\n7 min read\nHubble Survey Sets Up Roman\u2019s Future Look Near Milky Way\u2019s Center\narticle\n2 days ago\n5 min read\nNASA\u2019s Roman Poised to Transform Hunt for Elusive Neutron Stars\narticle\n7 days ago\n4 min read\nFor NASA\u2019s TESS, Stellar Eclipses Shed Light on Possible New Worlds\narticle\n1 week ago\nHighlights\n2 min read\nODYSSEY:\u00a0NASA\u00a0Analyzing\u00a0Bacteria in\u00a0Space, Simulated\u00a0Microgravity\narticle\n14 hours ago\n3 min read\nJoint Earth Observation Mission Quality Assessment Framework \u2013 Optical Guidelines Documents Released\narticle\n1 day ago\n7 min read\nHubble Survey Sets Up Roman\u2019s Future Look Near Milky Way\u2019s Center\narticle\n2 days ago\nHighlights\n3 min read\nMeet the Fleet: NASA Armstrong Continues Legacy of Flight Research\narticle\n5 days ago\n6 min read\nCornell Students Aid NASA with Drone Safety in Sky\narticle\n6 days ago\n4 min read\nD-Site\narticle\n1 week ago\nHighlights\n4 min read\nHello Universe: NASA\u2019s Next-Gen Space Processor Undergoes Testing\narticle\n13 hours ago\n3 min read\nI Am Artemis: Kathleen Harmon\narticle\n13 hours ago\n1 min read\nAmendment 56: D.6 APRA and D.7 SAT Final Text and Due Dates\narticle\n4 days ago\nFeatured\n4 min read\nSpace Out This Summer with Variety of NASA STEM Activities\narticle\n2 weeks ago\nFeatured\n3 min read\nNASA, Industry Advance High Performance Spaceflight Computing\narticle\n4 days ago\n3 min read\nIndustry Moon Lander Training Cabin Lands at NASA for Artemis\narticle\n5 days ago\n6 min read\nCornell Students Aid NASA with Drone Safety in Sky\narticle\n6 days ago\nHighlights\n11 min read\nLa NASA anuncia la cobertura de la misi\u00f3n lunar Artemis II\narticle\n2 months ago\n15 min read\nAgenda diaria de la misi\u00f3n a la Luna de Artemis\u00a0II de la NASA\narticle\n2 months ago\n6 min read\nLa NASA refuerza Artemis: a\u00f1ade una misi\u00f3n y perfecciona su arquitectura general\narticle\n2 months ago\nArtemis\nArtemis\nUnder Artemis, NASA will send astronauts on increasingly difficult missions to explore more of the Moon for scientific discovery, economic benefits, and to build on our foundation for the first crewed missions to Mars.\nQuick Facts\nArtemis II, the first crewed Artemis flight, marks a key step toward long\u2011term return to the Moon and future missions to Mars.\nDuring Artemis I, the SLS (Space Launch System), roared into the night sky and sent the Orion spacecraft on a 1.4-million-mile journey beyond the Moon and back.\nNASA, in coordination with the U.S. Department of State and seven other initial signatory nations, established the Artemis Accords in 2020.\nStrengthening Artemis\nTo achieve the national goal of landing American astronauts on the surface of the Moon and maintaining U.S. superiority in exploration and discovery, NASA is increasing its cadence of missions under the Artemis program, standardizing the SLS (Space Launch System) rocket configuration, and adding a new mission.\nArtemis Missions\nabout Strengthening Artemis\nArtemis News\nMore Artemis News\nArticle\n3 Min Read\nI Am Artemis: Kathleen Harmon\nArticle\n2 Min Read\nNicholas Houghton: Engineering Crew Safety for NASA\u2019s Artemis Missions\nArticle\n3 Min Read\nI Am Artemis: Anton Kiriwas\nArticle\n4 Min Read\nNASA Fuel Cell Tests Pave Way for Energy Storage on Moon\n61 Min Read\nArtemis II: Backup Crew\n3 Min Read\nNASA Welcomes Paraguay as 67th Artemis Accords Signatory\nArticle\n3 Min Read\nIndustry Moon Lander Training Cabin Lands at NASA for Artemis\nArticle\n3 Min Read\nNASA Welcomes Ireland as Newest Artemis Accords Signatory\nArticle\nLunar Exploration\nLunar Discovery\nMoon to Mars\nLunar Exploration\nThe Moon is a 4.5-billion-year-old time capsule.\nWe\u2019re going back to the Moon for scientific discovery, economic benefits, and inspiration for a new generation of explorers. While maintaining American leadership in exploration, we will build a global alliance and explore deep space for the benefit of all.\nEarth's Moon\nOn flight day six of the Artemis I mission, the Orion spacecraft used its optical navigation camera to snap this black-and-white photo of the Moon.\nNASA\nLunar Discovery\nThe Moon holds clues to the evolution of Earth, the planets, and the Sun.\nThrough Artemis, NASA will address high priority science questions, focusing on those that are best accomplished by on-site human explorers on and around the Moon and Mars by using robotic surface and orbiting systems.\nArtemis Science\nArtemis geology training lead at Johnson Space Center in Houston, Cindy Evans (left) and NASA astronaut Christina Koch study geologic features in Iceland during Artemis II crew geology training in August 2024.\nNASA/Robert Markowitz\nMoon to Mars\nLike the Moon, Mars is a rich destination for scientific discovery.\nMars remains our horizon goal for human exploration because it is one of the only other places we know where life may have existed in the solar system. What we learn about the Red Planet will tell us more about our Earth\u2019s past and future, and may help answer whether life exists beyond our home planet.\nHumans on Mars\nIllustration of an astronaut on Mars using a remote control drone to inspect a nearby cliff.\nNASA\nMissions\nArtemis I\nLaunched in 2022, Artemis I was the first in a series of increasingly complex missions that will enable human exploration at the Moon and future missions to Mars.\nArtemis II\nThe first crewed Artemis flight marks a key step toward long\u2011term return to the Moon and future missions to Mars.\nArtemis III\nScheduled for 2027, this new demonstration mission in low Earth orbit will test one or both commercial landers from SpaceX and Blue Origin, respectively.\nArtemis IV\nNASA continues to target early 2028 for the first Artemis lunar landing, a date that has remained unchanged since mid\u20112025. After reaching lunar orbit, the crew will transfer from Orion to a commercial lunar lander for their descent to the Moon\u2019s surface.\nArtemis V\nUsing the standard SLS (Space Launch System) rocket configuration, NASA expects to launch this lunar surface mission by late 2028, with subsequent missions planned roughly once per year.\nOur Artemis II Crew\nMeet the astronauts who ventured around the Moon on Artemis II, the first crewed flight aboard NASA\u2019s human deep space capabilities, paving the way for future lunar surface missions.\nForging New Frontiers\nabout Our Artemis II Crew\nMedia Resources\nArtemis II Press Kit\nArtemis II Reference Guide\nArtemis II Resources for Media\nSpacecraft\nRocket\nGround Systems\nLunar Landers\nSpacesuits &amp; Rovers\nLunar Delivery\nGateway\nArtemis Partners\nCarrying Humanity to the Moon\nOrion is developed to be capable of sending astronauts to the Moon and is a crucial step toward eventually sending crews on to Mars.\nThe Orion spacecraft will serve as the exploration vehicle that will carry and sustain the crew on Artemis missions to the Moon and return them safely to Earth. Orion will launch on NASA\u2019s new heavy-lift rocket, the SLS (Space Launch System).\nAbout Orion\nThe full Moon is seen behind NASA\u2019s Artemis II SLS (Space Launch System) rocket and Orion spacecraft, standing atop a mobile launcher at Launch Complex 39B, Sunday, Feb. 1, 2026, at Kennedy Space Center in Florida.\nNASA/John Kraus\nA Single Launch\nNASA\u2019s Space Launch System (SLS) offers more payload mass, volume, and departure energy than any other single rocket.\nCombining power and capability, NASA\u2019s SLS (Space Launch System) rocket is part of NASA\u2019s backbone for deep space exploration and Artemis. SLS is the only rocket that can send Orion, astronauts, and cargo directly to the Moon in a single launch.\nAbout the Space Launch System\nClouds and the Sun illuminate the sky on Wednesday, Jan. 28, 2026, as NASA\u2019s Artemis II SLS (Space Launch System) rocket and Orion spacecraft stand vertical at Launch Complex 39B at Kennedy Space Center in Florida.\nNASA/Cory S. Huston\nThe Infrastructure\nPreparing the infrastructure to support NASA\u2019s SLS (Space Launch System) rocket and Orion spacecraft.\nExploration Ground Systems, based at Kennedy Space Center in Florida, develops and operates the systems and facilities needed to process, launch, and recover rockets and spacecraft for NASA\u2019s Artemis missions.\nAbout Exploration Ground Systems\nTechnicians with NASA\u2019s Exploration Ground Systems team prepare to attach a crane to lift and secure NASA\u2019s Orion spacecraft on top of the SLS (Space Launch System) rocket in High Bay 3 of the Vehicle Assembly Building at Kennedy Space Center in Florida on Friday, Oct. 17, 2025.\nNASA/Amber Jean Notvest\nDelivering Crew, Cargo to the Lunar Frontier\nWorking with American industry to send crew, cargo, and supplies to the Moon.\nNASA is working with industry to develop the human landing systems, or next-generation landers, that will safely carry Artemis astronauts from lunar orbit to the\u2002Moon\u2019s surface and back for future crewed exploration of the Moon.\nAbout Lunar Landers\nArtist concept of SpaceX\u2019s Starship Human Landing System (HLS) on the Moon.\nSpaceX\nMobility for Every Mission\nProviding spacesuit capabilities and surface mobility systems for humanity\u2019s return to the Moon.\nThe Extravehicular Activity and Human Surface Mobility Program serves as NASA\u2019s program to develop next-generation spacesuits, human-rated rovers, tools, and the spacewalk support systems that will enable astronauts to survive and work outside the confines of a spacecraft to explore on and around the Moon.\nAbout Spacesuits &amp; Rovers\nIllustration of Artemis astronauts working on the Moon.\nNASA\nLanding on the Moon\nWorking with American companies to deliver science and technology to the Moon\u2019s surface.\nThe Commercial Lunar Payload Services (CLPS) initiative allows rapid acquisition of lunar delivery services from commercial vendors to send NASA science and technology payloads, enabling industry growth and supporting long-term lunar exploration. The CLPS model offers a unique opportunity to test and refine technologies and integrate systems that will provide insight for future crewed missions to the Moon.\nAbout Commercial Lunar Payload Services\nCarrying a suite of NASA science and technology, Firefly Aerospace\u2019s Blue Ghost Mission 1 successfully landed at 3:34 a.m. EST on Sunday, March 2, 2025, near a volcanic feature called Mons Latreille within Mare Crisium, a more than 300-mile-wide basin located in the northeast quadrant of the Moon\u2019s near side.\nFirefly Aerospace\nDeep Space Exploration\nHumanity\u2019s first space station around the Moon.\nGateway is central to the NASA-led Artemis missions to return to the Moon for scientific discovery and chart a path for the first human missions to Mars and beyond. The small space station will be a multi-purpose outpost supporting lunar surface missions, science in lunar orbit, and human exploration further into the cosmos.\nAbout Gateway\nGateway\u2019s HALO (Habitation and Logistics Outpost) at Northrop Grumman\u2019s facility in Gilbert, Arizona, on April 4, 2025, shortly after its arrival from Thales Alenia Space in Turin, Italy.\nNASA/Josh Valcarcel\nA Lunar Economy\nMen and women across America and around the world are building the systems to support missions to the Moon, Mars, and beyond.\nSince its inception, every state in America has made a contribution to the success of NASA\u2019s Artemis campaign, with companies hard at work on innovations that will help establish a long-term human presence at the Moon. These missions are critical to an expanding space economy, fueling new industries and technologies, supporting job growth, and furthering the demand for a highly skilled workforce.\nAbout Artemis Partners\nNASA\u2019s Artemis II Space Launch System (SLS) rocket and Orion spacecraft, secured to the mobile launcher, make the 4.2 mile journey toward Launch Pad 39B, Saturday, Jan. 17, 2026, at Kennedy Space Center in Florida.\nNASA/Keegan Barber\nThe Artemis Accords\nNASA, in coordination with the U.S. Department of State and seven other initial signatory nations, established the Artemis Accords in 2020. Now with more than 60 signatories, the Artemis Accords provide a common set of principles to enhance the governance of the civil exploration and use of outer space as many countries and private companies conduct missions and operations around the Moon.\nCivil Space Exploration\nabout The Artemis Accords\nLearning Resources\nJoin Artemis\nFind your place in space.\nMake, launch, compete and learn. Find your favorite way to be part of the Artemis mission.\nStart Exploring\nabout Join Artemis\nKeep Exploring\nDiscover More\nHumans In Space\nDestinations\nAstronauts\nLiving in Space\nWas this page helpful?\n\u0394\nWas this page helpful?\nYes\nNo\n\u00d7"}</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-05-08T22:41:52.575799</t>
+          <t>2026-05-13T04:49:15.985350</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>263af9bc-aad4-4bfb-ac49-cdc2f0fe5c4a</t>
+          <t>47843ecb-74e5-41c6-a654-58ed2eb4b677</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ranjithagowda9801@gmail.com</t>
+          <t>sahanashaiva01@gmail.com</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Revised_AI_MultiSummarizer_Plan (1).pdf</t>
+          <t>https://www.nasa.gov/humans-in-space/artemis/</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>file</t>
+          <t>url</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -585,22 +585,22 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>The project aims to create a sophisticated full-stack application that can process various content sources, including we...</t>
+          <t>The Artemis program is a series of missions designed to return humans to the Moon by 2028 and establish a sustainable pr</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>["AI", "Summarizer", "Content Intelligence", "React"]</t>
+          <t>["NASA", "Artemis", "Moon", "Mars"]</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>{"summary_concise": "The project involves developing a full-stack application that processes diverse content sources, extracts and summarizes text using AI, and provides sentiment analysis and reading metrics in a modern dashboard.", "summary_detailed": "The project aims to create a sophisticated full-stack application that can process various content sources, including website links and uploaded documents. The system will extract, clean, and summarize the text using AI, providing sentiment analysis and reading metrics in a modern dashboard. The application will have a modular grid UI, with each card having a specific responsibility, such as input module, metrics, main output, and visuals. The project will be implemented in several stages, including multi-source extraction, NLP core, API development, React Bento layout, and integration and analytics. The application will utilize various technologies, including React, Python, FastAPI, and NLTK, to achieve its goals. The project's technical requirements are well-defined, with a clear roadmap for implementation. The application's UI design is also well-planned, with a focus on modularity and ease of use.", "key_points": ["Full-stack application for content processing", "AI-powered text summarization and sentiment analysis", "Modular grid UI with specific responsibilities for each card", "Multi-source extraction and NLP core implementation", "API development and React Bento layout"], "important_insights": ["The application will utilize various technologies to achieve its goals", "The project's technical requirements are well-defined", "The application's UI design is focused on modularity and ease of use", "The project will be implemented in several stages"], "keywords": ["AI", "Summarizer", "Content Intelligence", "React", "Python", "NLTK", "Sentiment Analysis"], "metadata_insights": {"detected_topic": "Artificial Intelligence and Natural Language Processing", "reading_difficulty": "Advanced", "content_complexity": "High", "estimated_audience": "Technical professionals and developers", "category": "Technology and Software Development", "writing_style": "Technical and Informative"}, "tone_analysis": {"overall_tone": "Informative", "sentiment": "Neutral", "formality": "Formal", "confidence": "High", "confidence_score": 90, "sentiment_scores": {"positive": 20, "negative": 0, "neutral": 80}}, "source_text": "Multi-Format AI Summarizer\nAdvanced Content Intelligence Platform (URL, PDF, DOCX)\nProject Scope\nA sophisticated full-stack application that processes diverse content sources. Whether a\nuser provides a website link or uploads a document (PDF/Word), the system extracts,\ncleans, and summarizes the text using AI, providing sentiment analysis and reading\nmetrics in a modern dashboard.\nTechnical Requirements\nFrontend (React) Backend (Python)\n- React.js (Hooks &amp; Context) - FastAPI or Flask (REST API)\n- Tailwind CSS (Bento Layout) - PyPDF2 / pdfplumber (PDF)\n- React-Dropzone (File Uploads) - python-docx (Word Docs)\n- Recharts (Data Visuals) - BeautifulSoup4 (URL Scraping)\nAI &amp; Processing Workflow\n- NLTK / TextBlob (Summarization) - Axios for HTTP Requests\n- VADER (Sentiment Analysis) - FormData for File uploads\n- LangChain (Optional for better - LocalStorage for History\nchains)\nUI Design: Bento Dashboard\nThe UI is organized into a modular grid. Each \"card\" has a specific responsibility:\nInput Module: URL Toggle &amp; Drag-and-Drop File Zone\nMetrics: Word Count &amp; Read Time Main Output: AI\nGenerated Summary\n(Bulleted)\nVisuals: Sentiment Donut Chart\nImplementation Roadmap\n1 Multi-Source Extraction: Build a Python utility class that accepts a source (URL or\nFile). Use conditional logic to trigger the correct parser (BS4 for URLs, pdfplumber\nfor PDFs).\n2 NLP Core: Implement the summarization engine. Ensure the output is structured\n(Title, Key Points, Tone) so the React frontend can map it easily to cards.\n3 API Development: Create a POST endpoint that handles both JSON (for URLs) and\nMultipart/Form-Data (for file uploads).\n4 React Bento Layout: Build the grid using Tailwind `grid-cols`. Create a stateful\n\"Input Card\" that changes its UI based on whether the user wants to paste a link or\nupload a file.\n5 Integration &amp; Analytics: Connect the UI to the API. Implement the Sentiment\nChart and the history sidebar to save past results.\n"}</t>
+          <t>{"summary_concise": "NASA's Artemis program aims to send astronauts to the Moon and eventually to Mars, with the goal of establishing a sustainable presence on the lunar surface and beyond.", "summary_detailed": "The Artemis program is a series of missions designed to return humans to the Moon by 2028 and establish a sustainable presence on the lunar surface. The program includes several missions, including Artemis I, II, and III, which will test the Space Launch System (SLS) rocket and the Orion spacecraft. The ultimate goal of the program is to send humans to Mars and establish a sustainable presence in the solar system. The program also includes the development of new technologies, such as lunar landers and spacesuits, and the establishment of a lunar economy. The Artemis Accords, a set of principles for the governance of civil space exploration, have been established to guide the program and ensure international cooperation.", "key_points": ["NASA's Artemis program aims to send astronauts to the Moon and eventually to Mars", "The program includes several missions, including Artemis I, II, and III", "The Space Launch System (SLS) rocket and the Orion spacecraft are being developed for the program", "The program includes the development of new technologies, such as lunar landers and spacesuits", "The Artemis Accords provide a framework for international cooperation and governance of civil space exploration"], "important_insights": ["The Artemis program is a critical step towards establishing a sustainable human presence in the solar system", "The program requires significant technological advancements, including the development of new propulsion systems and life support systems", "International cooperation and governance will be essential for the success of the program", "The program has the potential to drive economic growth and create new opportunities for scientific discovery and exploration"], "keywords": ["NASA", "Artemis", "Moon", "Mars", "Space Exploration", "SLS", "Orion", "Lunar Landers", "Spacesuits"], "metadata_insights": {"detected_topic": "Space Exploration", "reading_difficulty": "Intermediate", "content_complexity": "High", "estimated_audience": "Space enthusiasts and professionals", "category": "Aerospace and Defense", "writing_style": "Informative"}, "tone_analysis": {"overall_tone": "Informative", "sentiment": "Neutral", "formality": "Formal", "confidence": "High", "confidence_score": 90, "sentiment_scores": {"positive": 20, "negative": 0, "neutral": 80}}, "source_text": "Moon to Mars | NASA's Artemis Program - NASA\nSearch\nSuggested Searches\nClimate Change\nArtemis\nExpedition 64\nMars perseverance\nSpaceX Crew-2\nInternational Space Station\nView All Topics A-Z\nHome\nMissions\nHumans in Space\nEarth\nThe Solar System\nThe Universe\nScience\nAeronautics\nTechnology\nLearning Resources\nAbout NASA\nEspa\u00f1ol\nNews &amp; Events\nMultimedia\nNASA+\nFeatured\n2 min read\nStudying Pneumonia in Space for Heart Health on Earth\narticle\n5 days ago\n4 min read\nNASA Outlines Preliminary Artemis III Mission Plans\narticle\n5 days ago\n3 min read\nWhat\u2019s Up: May 2026 Skywatching Tips from NASA\narticle\n3 weeks ago\nBack\nMissions\nSearch All NASA Missions\nA to Z List of Missions\nUpcoming Launches and Landings\nSpaceships and Rockets\nCommunicating with Missions\nArtemis\nJames Webb Space Telescope\nHubble Space Telescope\nInternational Space Station\nOSIRIS-Rex\nHumans in Space\nWhy Go to Space\nAstronauts\nCommercial Space\nDestinations\nSpaceships and Rockets\nLiving in Space\nEarth\nExplore Earth Science\nClimate Change\nEarth, Our Planet\nEarth Science in Action\nEarth Multimedia\nEarth Data\nEarth Science Researchers\nThe Solar System\nThe Sun\nMercury\nVenus\nEarth\nThe Moon\nMars\nJupiter\nSaturn\nUranus\nNeptune\nPluto &amp; Dwarf Planets\nAsteroids, Comets &amp; Meteors\nThe Kuiper Belt\nThe Oort Cloud\nSkywatching\nThe Universe\nExoplanets\nThe Search for Life in the Universe\nStars\nGalaxies\nBlack Holes\nThe Big Bang\nDark Energy\nDark Matter\nScience\nEarth Science\nPlanetary Science\nAstrophysics &amp; Space Science\nThe Sun &amp; Heliophysics\nBiological &amp; Physical Sciences\nLunar Science\nCitizen Science\nAstromaterials\nAeronautics Research\nHuman Space Travel Research\nAeronautics\nScience in the Air\nNASA Aircraft\nFlight Research Innovation\nSupersonic Flight\nAir Traffic Solutions\nGreen Aviation Tech\nDrones &amp; You\nTechnology\nTechnology Transfer &amp; Spinoffs\nSpace Travel Technology\nTechnology Living in Space\nManufacturing and Materials\nRobotics\nScience Instruments\nComputing\nLearning Resources\nFor Kids and Students\nFor Educators\nFor Colleges and Universities\nFor Professionals\nScience for Everyone\nRequests for Exhibits, Artifacts, Speakers &amp; Flyovers\nSTEM Engagement at NASA\nAbout NASA\nNASA's Impacts\nCenters and Facilities\nDirectorates\nOrganizations\nPeople of NASA\nCareers\nInternships\nOur History\nDoing Business with NASA\nGet Involved\nContact\nNASA en Espa\u00f1ol\nCiencia\nAeron\u00e1utica\nCiencias Terrestres\nSistema Solar\nUniverso\nNews &amp; Events\nNews Releases\nRecently Published\nVideo Series on NASA+\nPodcasts &amp; Audio\nBlogs\nNewsletters\nSocial Media\nMedia Resources\nEvents\nUpcoming Launches &amp; Landings\nVirtual Guest Program\nMultimedia\nNASA+\nImages\nNASA Live\nNASA Apps\nPodcasts\nImage of the Day\ne-Books\nInteractives\nSTEM Multimedia\nNASA Brand &amp; Usage Guidelines\nFeatured\n3 min read\nHubble Sights Galaxy in Transition\narticle\n3 days ago\n3 min read\nNASA\u2019s Planet-Hunting TESS Reveals Dazzling Night Sky\narticle\n5 days ago\n6 min read\nNASA\u2019s Perseverance Rover Snaps Selfie in Mars\u2019 Western Frontier\narticle\n6 days ago\nHighlights\n2 min read\nStudying Pneumonia in Space for Heart Health on Earth\narticle\n5 days ago\n3 min read\nNASA\u2019s Simulated Mars Mission Marks 200 Days Inside Habitat\narticle\n2 weeks ago\n2 min read\nNASA Astronaut to Answer Questions from Students in Florida\narticle\n2 weeks ago\nHighlights\n10 min read\nHelio and You: Seasons on Earth, Mars, and Beyond\narticle\n3 days ago\n3 min read\nPicturing Earth in a New Light\narticle\n3 days ago\n5 min read\nNASA Knows: The Ozone Hole\narticle\n4 days ago\nHighlights\n10 min read\nHelio and You: Seasons on Earth, Mars, and Beyond\narticle\n3 days ago\n2 min read\nNASA Draws on Industry for Mars Telecommunications Network\narticle\n4 days ago\n6 min read\nNASA\u2019s Perseverance Rover Snaps Selfie in Mars\u2019 Western Frontier\narticle\n6 days ago\nFeatured\n10 min read\nHelio and You: Seasons on Earth, Mars, and Beyond\narticle\n3 days ago\n3 min read\nHubble Sights Galaxy in Transition\narticle\n3 days ago\n3 min read\nNASA\u2019s Planet-Hunting TESS Reveals Dazzling Night Sky\narticle\n5 days ago\nHighlights\n10 min read\nHelio and You: Seasons on Earth, Mars, and Beyond\narticle\n3 days ago\n2 min read\nAmendment 57: D.3 AGIGO: IXPE and NICER General Observer Second Opportunity in ROSES-25\narticle\n3 days ago\n3 min read\nHubble Sights Galaxy in Transition\narticle\n3 days ago\nHighlights\n3 min read\nMeet the Fleet: NASA Armstrong Continues Legacy of Flight Research\narticle\n1 week ago\n6 min read\nCornell Students Aid NASA with Drone Safety in Sky\narticle\n2 weeks ago\n4 min read\nD-Site\narticle\n2 weeks ago\nHighlights\n3 min read\nPicturing Earth in a New Light\narticle\n3 days ago\n2 min read\nNASA Draws on Industry for Mars Telecommunications Network\narticle\n4 days ago\n3 min read\nNASA-Supported\u00a0Space Tech\u00a0Advances\u00a0Earthly\u00a0Construction\narticle\n5 days ago\nFeatured\n4 min read\nSpace Out This Summer with Variety of NASA STEM Activities\narticle\n2 weeks ago\nFeatured\n2 min read\nNASA Draws on Industry for Mars Telecommunications Network\narticle\n4 days ago\n2 min read\nNASA, Industry Prepare Cryogenic Fuel Technology Demo\narticle\n4 days ago\n3 min read\nNASA-Supported\u00a0Space Tech\u00a0Advances\u00a0Earthly\u00a0Construction\narticle\n5 days ago\nHighlights\n11 min read\nLa NASA anuncia la cobertura de la misi\u00f3n lunar Artemis II\narticle\n2 months ago\n15 min read\nAgenda diaria de la misi\u00f3n a la Luna de Artemis\u00a0II de la NASA\narticle\n2 months ago\n6 min read\nLa NASA refuerza Artemis: a\u00f1ade una misi\u00f3n y perfecciona su arquitectura general\narticle\n3 months ago\nArtemis\nArtemis\nUnder Artemis, NASA will send astronauts on increasingly difficult missions to explore more of the Moon for scientific discovery, economic benefits, and to build on our foundation for the first crewed missions to Mars.\nQuick Facts\nArtemis II, the first crewed Artemis flight, marks a key step toward long\u2011term return to the Moon and future missions to Mars.\nDuring Artemis I, the SLS (Space Launch System), roared into the night sky and sent the Orion spacecraft on a 1.4-million-mile journey beyond the Moon and back.\nNASA, in coordination with the U.S. Department of State and seven other initial signatory nations, established the Artemis Accords in 2020.\nStrengthening Artemis\nTo achieve the national goal of landing American astronauts on the surface of the Moon and maintaining U.S. superiority in exploration and discovery, NASA is increasing its cadence of missions under the Artemis program, standardizing the SLS (Space Launch System) rocket configuration, and adding a new mission.\nArtemis Missions\nabout Strengthening Artemis\nArtemis News\nMore Artemis News\nImage Article\n1 Min Read\nRise Goes to Washington\nArticle\n4 Min Read\nNASA Outlines Preliminary Artemis III Mission Plans\nArticle\n3 Min Read\nI Am Artemis: Kathleen Harmon\nArticle\n2 Min Read\nNicholas Houghton: Engineering Crew Safety for NASA\u2019s Artemis Missions\n3 Min Read\nI Am Artemis: Anton Kiriwas\nArticle\n4 Min Read\nNASA Fuel Cell Tests Pave Way for Energy Storage on Moon\nArticle\n61 Min Read\nArtemis II: Backup Crew\n3 Min Read\nNASA Welcomes Paraguay as 67th Artemis Accords Signatory\nArticle\nLunar Exploration\nLunar Discovery\nMoon to Mars\nLunar Exploration\nThe Moon is a 4.5-billion-year-old time capsule.\nWe\u2019re going back to the Moon for scientific discovery, economic benefits, and inspiration for a new generation of explorers. While maintaining American leadership in exploration, we will build a global alliance and explore deep space for the benefit of all.\nEarth's Moon\nOn flight day six of the Artemis I mission, the Orion spacecraft used its optical navigation camera to snap this black-and-white photo of the Moon.\nNASA\nLunar Discovery\nThe Moon holds clues to the evolution of Earth, the planets, and the Sun.\nThrough Artemis, NASA will address high priority science questions, focusing on those that are best accomplished by on-site human explorers on and around the Moon and Mars by using robotic surface and orbiting systems.\nArtemis Science\nArtemis geology training lead at Johnson Space Center in Houston, Cindy Evans (left) and NASA astronaut Christina Koch study geologic features in Iceland during Artemis II crew geology training in August 2024.\nNASA/Robert Markowitz\nMoon to Mars\nLike the Moon, Mars is a rich destination for scientific discovery.\nMars remains our horizon goal for human exploration because it is one of the only other places we know where life may have existed in the solar system. What we learn about the Red Planet will tell us more about our Earth\u2019s past and future, and may help answer whether life exists beyond our home planet.\nHumans on Mars\nIllustration of an astronaut on Mars using a remote control drone to inspect a nearby cliff.\nNASA\nMissions\nArtemis I\nLaunched in 2022, Artemis I was the first in a series of increasingly complex missions that will enable human exploration at the Moon and future missions to Mars.\nArtemis II\nThe first crewed Artemis flight marks a key step toward long\u2011term return to the Moon and future missions to Mars.\nArtemis III\nScheduled for 2027, this new demonstration mission in low Earth orbit will test one or both commercial landers from SpaceX and Blue Origin, respectively.\nArtemis IV\nNASA continues to target early 2028 for the first Artemis lunar landing, a date that has remained unchanged since mid\u20112025. After reaching lunar orbit, the crew will transfer from Orion to a commercial lunar lander for their descent to the Moon\u2019s surface.\nArtemis V\nUsing the standard SLS (Space Launch System) rocket configuration, NASA expects to launch this lunar surface mission by late 2028, with subsequent missions planned roughly once per year.\nOur Artemis II Crew\nMeet the astronauts who ventured around the Moon on Artemis II, the first crewed flight aboard NASA\u2019s human deep space capabilities, paving the way for future lunar surface missions.\nForging New Frontiers\nabout Our Artemis II Crew\nMedia Resources\nArtemis II Press Kit\nArtemis II Reference Guide\nArtemis II Resources for Media\nSpacecraft\nRocket\nGround Systems\nLunar Landers\nSpacesuits &amp; Rovers\nLunar Delivery\nGateway\nArtemis Partners\nCarrying Humanity to the Moon\nOrion is developed to be capable of sending astronauts to the Moon and is a crucial step toward eventually sending crews on to Mars.\nThe Orion spacecraft will serve as the exploration vehicle that will carry and sustain the crew on Artemis missions to the Moon and return them safely to Earth. Orion will launch on NASA\u2019s new heavy-lift rocket, the SLS (Space Launch System).\nAbout Orion\nThe full Moon is seen behind NASA\u2019s Artemis II SLS (Space Launch System) rocket and Orion spacecraft, standing atop a mobile launcher at Launch Complex 39B, Sunday, Feb. 1, 2026, at Kennedy Space Center in Florida.\nNASA/John Kraus\nA Single Launch\nNASA\u2019s Space Launch System (SLS) offers more payload mass, volume, and departure energy than any other single rocket.\nCombining power and capability, NASA\u2019s SLS (Space Launch System) rocket is part of NASA\u2019s backbone for deep space exploration and Artemis. SLS is the only rocket that can send Orion, astronauts, and cargo directly to the Moon in a single launch.\nAbout the Space Launch System\nClouds and the Sun illuminate the sky on Wednesday, Jan. 28, 2026, as NASA\u2019s Artemis II SLS (Space Launch System) rocket and Orion spacecraft stand vertical at Launch Complex 39B at Kennedy Space Center in Florida.\nNASA/Cory S. Huston\nThe Infrastructure\nPreparing the infrastructure to support NASA\u2019s SLS (Space Launch System) rocket and Orion spacecraft.\nExploration Ground Systems, based at Kennedy Space Center in Florida, develops and operates the systems and facilities needed to process, launch, and recover rockets and spacecraft for NASA\u2019s Artemis missions.\nAbout Exploration Ground Systems\nTechnicians with NASA\u2019s Exploration Ground Systems team prepare to attach a crane to lift and secure NASA\u2019s Orion spacecraft on top of the SLS (Space Launch System) rocket in High Bay 3 of the Vehicle Assembly Building at Kennedy Space Center in Florida on Friday, Oct. 17, 2025.\nNASA/Amber Jean Notvest\nDelivering Crew, Cargo to the Lunar Frontier\nWorking with American industry to send crew, cargo, and supplies to the Moon.\nNASA is working with industry to develop the human landing systems, or next-generation landers, that will safely carry Artemis astronauts from lunar orbit to the\u2002Moon\u2019s surface and back for future crewed exploration of the Moon.\nAbout Lunar Landers\nArtist concept of SpaceX\u2019s Starship Human Landing System (HLS) on the Moon.\nSpaceX\nMobility for Every Mission\nProviding spacesuit capabilities and surface mobility systems for humanity\u2019s return to the Moon.\nThe Extravehicular Activity and Human Surface Mobility Program serves as NASA\u2019s program to develop next-generation spacesuits, human-rated rovers, tools, and the spacewalk support systems that will enable astronauts to survive and work outside the confines of a spacecraft to explore on and around the Moon.\nAbout Spacesuits &amp; Rovers\nIllustration of Artemis astronauts working on the Moon.\nNASA\nLanding on the Moon\nWorking with American companies to deliver science and technology to the Moon\u2019s surface.\nThe Commercial Lunar Payload Services (CLPS) initiative allows rapid acquisition of lunar delivery services from commercial vendors to send NASA science and technology payloads, enabling industry growth and supporting long-term lunar exploration. The CLPS model offers a unique opportunity to test and refine technologies and integrate systems that will provide insight for future crewed missions to the Moon.\nAbout Commercial Lunar Payload Services\nCarrying a suite of NASA science and technology, Firefly Aerospace\u2019s Blue Ghost Mission 1 successfully landed at 3:34 a.m. EST on Sunday, March 2, 2025, near a volcanic feature called Mons Latreille within Mare Crisium, a more than 300-mile-wide basin located in the northeast quadrant of the Moon\u2019s near side.\nFirefly Aerospace\nDeep Space Exploration\nHumanity\u2019s first space station around the Moon.\nGateway is central to the NASA-led Artemis missions to return to the Moon for scientific discovery and chart a path for the first human missions to Mars and beyond. The small space station will be a multi-purpose outpost supporting lunar surface missions, science in lunar orbit, and human exploration further into the cosmos.\nAbout Gateway\nGateway\u2019s HALO (Habitation and Logistics Outpost) at Northrop Grumman\u2019s facility in Gilbert, Arizona, on April 4, 2025, shortly after its arrival from Thales Alenia Space in Turin, Italy.\nNASA/Josh Valcarcel\nA Lunar Economy\nMen and women across America and around the world are building the systems to support missions to the Moon, Mars, and beyond.\nSince its inception, every state in America has made a contribution to the success of NASA\u2019s Artemis campaign, with companies hard at work on innovations that will help establish a long-term human presence at the Moon. These missions are critical to an expanding space economy, fueling new industries and technologies, supporting job growth, and furthering the demand for a highly skilled workforce.\nAbout Artemis Partners\nNASA\u2019s Artemis II Space Launch System (SLS) rocket and Orion spacecraft, secured to the mobile launcher, make the 4.2 mile journey toward Launch Pad 39B, Saturday, Jan. 17, 2026, at Kennedy Space Center in Florida.\nNASA/Keegan Barber\nThe Artemis Accords\nNASA, in coordination with the U.S. Department of State and seven other initial signatory nations, established the Artemis Accords in 2020. Now with more than 60 signatories, the Artemis Accords provide a common set of principles to enhance the governance of the civil exploration and use of outer space as many countries and private companies conduct missions and operations around the Moon.\nCivil Space Exploration\nabout The Artemis Accords\nLearning Resources\nJoin Artemis\nFind your place in space.\nMake, launch, compete and learn. Find your favorite way to be part of the Artemis mission.\nStart Exploring\nabout Join Artemis\nKeep Exploring\nDiscover More\nHumans In Space\nDestinations\nAstronauts\nLiving in Space\nWas this page helpful?\n\u0394\nWas this page helpful?\nYes\nNo\n\u00d7", "chat": [{"role": "user", "content": "what is this aout"}, {"role": "assistant", "content": "This document appears to be about NASA's Artemis program, which is a mission to return humans to the Moon and eventually send humans to Mars. The document provides an overview of the program, its goals, and its various components, including the Space Launch System (SLS) rocket, the Orion spacecraft, and the Gateway space station. It also discusses the program's progress, its international partnerships, and its plans for future missions."}]}</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-05-08T22:43:29.686445</t>
+          <t>2026-05-18T10:23:35.664726</t>
         </is>
       </c>
     </row>

</xml_diff>